<commit_message>
Sync changes for dataset
</commit_message>
<xml_diff>
--- a/datasets/IndicWikiQA-Tam_EN.xlsx
+++ b/datasets/IndicWikiQA-Tam_EN.xlsx
@@ -565,7 +565,7 @@
     <t>Which sweet, steamed dumpling is traditionally offered to Pillayar during his festival?</t>
   </si>
   <si>
-    <t>Modagam</t>
+    <t>Modak (Kozhukattai)</t>
   </si>
   <si>
     <t>What tiered, thematic doll display is a central tradition in Tamil households during Navaratri?</t>
@@ -1998,7 +1998,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2311,7 +2311,7 @@
     <col min="4" max="4" style="5" width="21.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -2339,7 +2339,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
@@ -2465,7 +2465,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="2" t="s">
         <v>38</v>
       </c>
@@ -2493,7 +2493,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="2" t="s">
         <v>41</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="2" t="s">
         <v>44</v>
       </c>
@@ -2521,7 +2521,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="2" t="s">
         <v>47</v>
       </c>
@@ -2535,7 +2535,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="2" t="s">
         <v>50</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="2" t="s">
         <v>53</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="2" t="s">
         <v>56</v>
       </c>

</xml_diff>